<commit_message>
Advocacy page, and lund, and more buses
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Published 2026-07-25 by BC Cycle Tourism Society.</t>
+          <t>Published 2026-07-26 by BC Cycle Tourism Society.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-07-25. https://bccycletourism.ca/research/</t>
+          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-07-26. https://bccycletourism.ca/research/</t>
         </is>
       </c>
     </row>
@@ -540,42 +540,49 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Of the 67 carriers here, 30 have had their bicycle policy checked against the operator's own material, 9 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
+          <t>There is no feed. The registry behind these files is kept by hand, assembled service by service from operator websites, regional transit schedules, tourism listings, ferry timetables, and telephone calls. It is a collection, not a census: we cannot know what we have missed, so treat every count as a floor, never a total.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Of the 67 carriers here, 30 have had their bicycle policy checked against the operator's own material, 9 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Where we have checked an operator specifically and found that it does not carry bicycles, that verdict is what the row publishes, and any policy text derived from the operator's own listing is suppressed. Those two do disagree for at least one carrier, whose published material still describes reserving a bicycle space. The checked answer is the one we stand behind.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Bicycle policies change, and this is the one place in our research where stale data has a physical cost. A route measurement that goes out of date is a mild embarrassment. A bicycle policy that goes out of date leaves somebody standing at a depot with a loaded bicycle and no way onto the bus. Check the last_verified column before you rely on a row, and confirm with the operator before you travel.</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Bicycle policies change, and this is the one place in our research where stale data has a physical cost. A route measurement that goes out of date is a mild embarrassment. A bicycle policy that goes out of date leaves somebody standing at a depot with a loaded bicycle and no way onto the bus. Check the last_verified column in the carriers file before you rely on a row, and confirm with the operator before you travel.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>We do not run any of these services. Operators change their routes, their seasons and their bicycle rules without telling us. Corrections are welcome and we would rather hear about a wrong row than not.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>The research here uses AI assistance (Claude models, Anthropic) for data collection, analysis, and writing. Feel free to ask for more details if you are interested.</t>
         </is>
@@ -1020,10 +1027,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="D9" t="n">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1151,7 +1158,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1417,7 +1424,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1819,6 +1826,11 @@
           <t>operator-checked</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>https://bccycletourism.ca/wwc/stop/42fea27c49/</t>
@@ -2084,7 +2096,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2621,6 +2633,11 @@
           <t>operator-checked</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr">
         <is>
           <t>https://bccycletourism.ca/wwc/stop/e9065ae25e/</t>
@@ -2995,12 +3012,17 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Roll on, free (2 bikes per car); Avoid rush hour; E-bikes OK</t>
+          <t>Roll on, free (bikes ride inside the cabin); 6 bikes per sailing at rush hour (weekdays 7–9:30 am and 3–6:30 pm; no limit other times); E-bikes OK (no charging on board); No trailers (185 cm max bike length)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>No trailers (185 cm max bike length)</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>preparation</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3010,7 +3032,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3269,6 +3291,11 @@
       <c r="I61" t="inlineStr">
         <is>
           <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -3757,7 +3784,7 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>What the operator does with a bicycle, in plain words. Blank where bikes_carried is unknown.</t>
+          <t>What the operator does with a bicycle, in plain words. Blank where bikes_carried is unknown. Where an operator runs more than one kind of service, this describes one of them; our trip planner shows mode-specific wording for each leg.</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3860,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>When a person last checked. Blank means we hold no date, which for some carriers means nobody has checked and for others means the check was not dated. Read it with policy_source.</t>
+          <t>When a person last checked this carrier against the operator's own material. Per-carrier: most rows carry the July 2026 vetting pass, carriers checked individually since then carry their own later dates. Blank means nobody has checked. Read it with policy_source.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add 10 new towns to to and fro
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -1027,10 +1027,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D9" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
quick fixes + research refresh: teal visited links site-wide, eager image preload, field notes dispatch teaser, transit numbers to aug 11 build, retire 7 route variants
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkuNDjmSEbdGEWN6Rhj5Do
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -462,7 +462,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Published 2026-07-26 by BC Cycle Tourism Society.</t>
+          <t>Published 2026-08-11 by BC Cycle Tourism Society.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-07-26. https://bccycletourism.ca/research/</t>
+          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-08-11. https://bccycletourism.ca/research/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update transit facts, fix bike url
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -547,7 +547,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Of the 67 carriers here, 30 have had their bicycle policy checked against the operator's own material, 9 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
+          <t>Of the 67 carriers here, 32 have had their bicycle policy checked against the operator's own material, 7 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Rides in the hold (boxed, bagged, or wrapped); Reserve bike spot</t>
+          <t>Luggage bay on the Prince Rupert route; Other routes: bagged or boxed (checked as luggage)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -900,7 +900,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1034,22 +1039,32 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>yes, with conditions</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rack on the bus, free (2 bikes · first come, first served); E-bikes OK</t>
+          <t>Front rack, no fee (2 bikes, first come; space not guaranteed); E-bikes under 25 kg only (lithium battery off the bike and carried on board)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>E-bikes under 25 kg only (lithium battery off the bike and carried on board)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">

</xml_diff>

<commit_message>
Dispatch #3 (August 2026): To and Fro feature, Trailside Buffet, smoke + mobile-mechanic how-tos, Be Prepared updates, dispatch page + email archive
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -513,7 +513,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carriers: 67 rows, 12 columns.</t>
+          <t>Carriers: 68 rows, 12 columns.</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Of the 67 carriers here, 32 have had their bicycle policy checked against the operator's own material, 7 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
+          <t>Of the 68 carriers here, 33 have had their bicycle policy checked against the operator's own material, 7 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1677,10 +1677,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D24" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2909,10 +2909,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D53" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -3213,35 +3213,65 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Victoria Harbour Ferry</t>
+          <t>Victoria Clipper</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Reserve ahead by phone (space very limited, first booked first served); $30 USD each way (about $41 CAD); Rides on the open deck (bags and accessories off; waiver at check-in)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Rides on the open deck (bags and accessories off; waiver at check-in)</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/f217a1bbde/</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://www.clippervacations.com</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>West Coast Launch</t>
+          <t>Victoria Harbour Ferry</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3250,10 +3280,10 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3263,189 +3293,159 @@
       <c r="I60" t="inlineStr">
         <is>
           <t>not-on-file</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/22a5ae41f3/</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>https://www.westcoastlaunch.com/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>West Coast Trail Express</t>
+          <t>West Coast Launch</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D61" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/5117c40285/</t>
+          <t>https://bccycletourism.ca/wwc/stop/22a5ae41f3/</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://trailbus.com/</t>
+          <t>https://www.westcoastlaunch.com/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>West Coast Transit System (Tofino/Ucluelet)</t>
+          <t>West Coast Trail Express</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>local-bus</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Rack on the bus, free (2 bikes · first come, first served); E-bikes OK</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>none</t>
+          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
+          <t>https://bccycletourism.ca/wwc/stop/5117c40285/</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.bctransit.com</t>
+          <t>https://trailbus.com/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>WestJet</t>
+          <t>West Coast Transit System (Tofino/Ucluelet)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>local-bus</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Box or sturdy bag required; Bike fee; No e-bikes</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Box or sturdy bag required; No e-bikes</t>
+          <t>Rack on the bus, free (2 bikes · first come, first served); E-bikes OK</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>none</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>listing-description</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/b5f48a88ff/</t>
+          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.westjet.com</t>
+          <t>https://www.bctransit.com</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Whistler Shuttle</t>
+          <t>WestJet</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D64" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -3454,12 +3454,17 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Book ahead (bikes carried with advance notice); Bike fee</t>
+          <t>Box or sturdy bag required; Bike fee; No e-bikes</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Box or sturdy bag required; No e-bikes</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>preparation</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3474,100 +3479,100 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/c7e12671ea/</t>
+          <t>https://bccycletourism.ca/wwc/stop/b5f48a88ff/</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.whistlershuttle.com</t>
+          <t>https://www.westjet.com</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Wilderness Seaplanes</t>
+          <t>Whistler Shuttle</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Book ahead (bikes carried with advance notice); Bike fee</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/c7e12671ea/</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>https://www.whistlershuttle.com</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Wilson's Transportation (BC Connector)</t>
+          <t>Wilderness Seaplanes</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Rides in the hold (bagged or boxed); $42 per bike (50 lb max); Reserve bike spot (recommended)</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/ca9171f28f/</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>https://wilsonstransportation.com/</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>YVR Skylynx</t>
+          <t>Wilson's Transportation (BC Connector)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3588,7 +3593,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Rides in the hold (bagged, wrapped, or boxed); First bike free; Reserve ahead (Squamish is reservation-only)</t>
+          <t>Rides in the hold (bagged or boxed); $42 per bike (50 lb max); Reserve bike spot (recommended)</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3608,38 +3613,91 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/49b1ded455/</t>
+          <t>https://bccycletourism.ca/wwc/stop/ca9171f28f/</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.yvrskylynx.com</t>
+          <t>https://wilsonstransportation.com/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>YVR Skylynx</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Rides in the hold (bagged, wrapped, or boxed); First bike free; Reserve ahead (Squamish is reservation-only)</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>preparation</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/49b1ded455/</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>https://www.yvrskylynx.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>Zeballos Expeditions (Zeballos Water Taxi)</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>water-taxi</t>
         </is>
       </c>
-      <c r="C68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D68" t="n">
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" t="n">
         <v>0</v>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
+      <c r="I69" t="inlineStr">
         <is>
           <t>not-on-file</t>
         </is>

</xml_diff>

<commit_message>
distance sort, chain street hints, GP cross-stamp reversal, research numbers   refresh
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -462,7 +462,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Published 2026-08-11 by BC Cycle Tourism Society.</t>
+          <t>Published 2026-09-02 by BC Cycle Tourism Society.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-08-11. https://bccycletourism.ca/research/</t>
+          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-09-02. https://bccycletourism.ca/research/</t>
         </is>
       </c>
     </row>

</xml_diff>